<commit_message>
update multiple files at revision time
</commit_message>
<xml_diff>
--- a/02_Basic_Excel_for_Data_Analytics/13P_sample_students_marks.xlsx
+++ b/02_Basic_Excel_for_Data_Analytics/13P_sample_students_marks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01 COURSES\Learn_Data_Analytics_by_CWH\02_Basic_Excel_for_Data_Analytics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{214B283B-F8BE-4689-AAFB-B01D51DA5A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{812BA5D0-F40D-41B7-8384-6124DD43C8D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Student Marks" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Student Marks'!$A$1:$I$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Student Marks'!$A$1:$I$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
@@ -230,15 +230,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -261,17 +267,72 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -279,243 +340,35 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="30">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="12">
     <dxf>
       <font>
         <b/>
         <i val="0"/>
         <strike/>
         <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color rgb="FFC00000"/>
       </font>
       <fill>
         <patternFill>
@@ -555,8 +408,53 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
         <strike/>
-        <color rgb="FFC00000"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
@@ -895,98 +793,100 @@
   <dimension ref="A1:I51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.54296875" customWidth="1"/>
-    <col min="2" max="3" width="14.36328125" customWidth="1"/>
-    <col min="4" max="4" width="18.36328125" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="14.36328125" customWidth="1"/>
-    <col min="8" max="8" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="17" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:9" ht="17.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="11" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="3">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="6">
         <v>43</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="6">
         <v>43</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="6">
         <v>46</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="6">
         <v>47</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="6">
         <v>53</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="7">
         <f>SUM(C2:G2)/500</f>
         <v>0.46400000000000002</v>
       </c>
-      <c r="I2" s="1" t="str">
+      <c r="I2" s="8" t="str">
         <f>IF(H2&gt;0.7,"pass","fail")</f>
         <v>fail</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>46</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>48</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>50</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="3">
         <v>49</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="3">
         <v>56</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="4">
         <f t="shared" ref="H3:H51" si="0">SUM(C3:G3)/500</f>
         <v>0.498</v>
       </c>
@@ -996,28 +896,28 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>49</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>53</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>54</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <v>51</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="3">
         <v>59</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="4">
         <f t="shared" si="0"/>
         <v>0.53200000000000003</v>
       </c>
@@ -1027,28 +927,28 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="3">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="3">
         <v>52</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>58</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <v>58</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="3">
         <v>53</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="3">
         <v>62</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="4">
         <f t="shared" si="0"/>
         <v>0.56599999999999995</v>
       </c>
@@ -1058,28 +958,28 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="3">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="3">
         <v>55</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>63</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <v>62</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="3">
         <v>55</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="3">
         <v>65</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="4">
         <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
@@ -1089,28 +989,28 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" s="3">
+      <c r="A7" s="2">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="3">
         <v>58</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>68</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="3">
         <v>66</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="3">
         <v>57</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="3">
         <v>68</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="4">
         <f t="shared" si="0"/>
         <v>0.63400000000000001</v>
       </c>
@@ -1120,28 +1020,28 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" s="3">
+      <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="3">
         <v>61</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <v>73</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="3">
         <v>70</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="3">
         <v>59</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="3">
         <v>71</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="4">
         <f t="shared" si="0"/>
         <v>0.66800000000000004</v>
       </c>
@@ -1151,28 +1051,28 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="3">
+      <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="3">
         <v>64</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="3">
         <v>78</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="3">
         <v>74</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="3">
         <v>61</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="3">
         <v>74</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="4">
         <f t="shared" si="0"/>
         <v>0.70199999999999996</v>
       </c>
@@ -1182,28 +1082,28 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" s="3">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="3">
         <v>67</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <v>83</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <v>78</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="3">
         <v>63</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="3">
         <v>77</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="4">
         <f t="shared" si="0"/>
         <v>0.73599999999999999</v>
       </c>
@@ -1213,28 +1113,28 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="3">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="3">
         <v>70</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="3">
         <v>88</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <v>82</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="3">
         <v>65</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="3">
         <v>80</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="4">
         <f t="shared" si="0"/>
         <v>0.77</v>
       </c>
@@ -1244,28 +1144,28 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="3">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="3">
         <v>73</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="3">
         <v>93</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="3">
         <v>86</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="3">
         <v>67</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="3">
         <v>83</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="4">
         <f t="shared" si="0"/>
         <v>0.80400000000000005</v>
       </c>
@@ -1275,28 +1175,28 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A13" s="3">
+      <c r="A13" s="2">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="3">
         <v>76</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="3">
         <v>98</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="3">
         <v>90</v>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="3">
         <v>69</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="3">
         <v>86</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="4">
         <f t="shared" si="0"/>
         <v>0.83799999999999997</v>
       </c>
@@ -1306,28 +1206,28 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="3">
+      <c r="A14" s="2">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C14" s="3">
         <v>79</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="3">
         <v>40</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="3">
         <v>94</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="3">
         <v>71</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14" s="3">
         <v>89</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="4">
         <f t="shared" si="0"/>
         <v>0.746</v>
       </c>
@@ -1337,28 +1237,28 @@
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="3">
+      <c r="A15" s="2">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C15" s="3">
         <v>82</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="3">
         <v>45</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="3">
         <v>98</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="3">
         <v>73</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="3">
         <v>92</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="4">
         <f t="shared" si="0"/>
         <v>0.78</v>
       </c>
@@ -1368,28 +1268,28 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="3">
+      <c r="A16" s="2">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C16" s="3">
         <v>85</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="3">
         <v>50</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="3">
         <v>43</v>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="3">
         <v>75</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16" s="3">
         <v>95</v>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="4">
         <f t="shared" si="0"/>
         <v>0.69599999999999995</v>
       </c>
@@ -1399,28 +1299,28 @@
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A17" s="3">
+      <c r="A17" s="2">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="3">
         <v>88</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="3">
         <v>55</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="3">
         <v>47</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="3">
         <v>77</v>
       </c>
-      <c r="G17" s="4">
+      <c r="G17" s="3">
         <v>98</v>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="4">
         <f t="shared" si="0"/>
         <v>0.73</v>
       </c>
@@ -1430,28 +1330,28 @@
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A18" s="3">
+      <c r="A18" s="2">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="4">
+      <c r="C18" s="3">
         <v>91</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="3">
         <v>60</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="3">
         <v>51</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="3">
         <v>79</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18" s="3">
         <v>50</v>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="4">
         <f t="shared" si="0"/>
         <v>0.66200000000000003</v>
       </c>
@@ -1461,28 +1361,28 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A19" s="3">
+      <c r="A19" s="2">
         <v>18</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="3">
         <v>94</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="3">
         <v>65</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="3">
         <v>55</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="3">
         <v>81</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19" s="3">
         <v>53</v>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="4">
         <f t="shared" si="0"/>
         <v>0.69599999999999995</v>
       </c>
@@ -1492,28 +1392,28 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A20" s="3">
+      <c r="A20" s="2">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C20" s="3">
         <v>97</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="3">
         <v>70</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="3">
         <v>59</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="3">
         <v>83</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G20" s="3">
         <v>56</v>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="4">
         <f t="shared" si="0"/>
         <v>0.73</v>
       </c>
@@ -1523,28 +1423,28 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A21" s="3">
+      <c r="A21" s="2">
         <v>20</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="3">
         <v>100</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="3">
         <v>75</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="3">
         <v>63</v>
       </c>
-      <c r="F21" s="4">
+      <c r="F21" s="3">
         <v>85</v>
       </c>
-      <c r="G21" s="4">
+      <c r="G21" s="3">
         <v>59</v>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="4">
         <f t="shared" si="0"/>
         <v>0.76400000000000001</v>
       </c>
@@ -1554,28 +1454,28 @@
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A22" s="3">
+      <c r="A22" s="2">
         <v>21</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="3">
         <v>42</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="3">
         <v>80</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22" s="3">
         <v>67</v>
       </c>
-      <c r="F22" s="4">
+      <c r="F22" s="3">
         <v>87</v>
       </c>
-      <c r="G22" s="4">
+      <c r="G22" s="3">
         <v>62</v>
       </c>
-      <c r="H22" s="5">
+      <c r="H22" s="4">
         <f t="shared" si="0"/>
         <v>0.67600000000000005</v>
       </c>
@@ -1585,28 +1485,28 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A23" s="3">
+      <c r="A23" s="2">
         <v>22</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C23" s="4">
+      <c r="C23" s="3">
         <v>45</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="3">
         <v>85</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23" s="3">
         <v>71</v>
       </c>
-      <c r="F23" s="4">
+      <c r="F23" s="3">
         <v>89</v>
       </c>
-      <c r="G23" s="4">
+      <c r="G23" s="3">
         <v>65</v>
       </c>
-      <c r="H23" s="5">
+      <c r="H23" s="4">
         <f t="shared" si="0"/>
         <v>0.71</v>
       </c>
@@ -1616,28 +1516,28 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A24" s="3">
+      <c r="A24" s="2">
         <v>23</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C24" s="4">
+      <c r="C24" s="3">
         <v>48</v>
       </c>
-      <c r="D24" s="4">
+      <c r="D24" s="3">
         <v>90</v>
       </c>
-      <c r="E24" s="4">
+      <c r="E24" s="3">
         <v>75</v>
       </c>
-      <c r="F24" s="4">
+      <c r="F24" s="3">
         <v>91</v>
       </c>
-      <c r="G24" s="4">
+      <c r="G24" s="3">
         <v>68</v>
       </c>
-      <c r="H24" s="5">
+      <c r="H24" s="4">
         <f t="shared" si="0"/>
         <v>0.74399999999999999</v>
       </c>
@@ -1647,28 +1547,28 @@
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A25" s="3">
+      <c r="A25" s="2">
         <v>24</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="3">
         <v>51</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="3">
         <v>95</v>
       </c>
-      <c r="E25" s="4">
+      <c r="E25" s="3">
         <v>79</v>
       </c>
-      <c r="F25" s="4">
+      <c r="F25" s="3">
         <v>93</v>
       </c>
-      <c r="G25" s="4">
+      <c r="G25" s="3">
         <v>71</v>
       </c>
-      <c r="H25" s="5">
+      <c r="H25" s="4">
         <f t="shared" si="0"/>
         <v>0.77800000000000002</v>
       </c>
@@ -1678,28 +1578,28 @@
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A26" s="3">
+      <c r="A26" s="2">
         <v>25</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C26" s="4">
+      <c r="C26" s="3">
         <v>54</v>
       </c>
-      <c r="D26" s="4">
+      <c r="D26" s="3">
         <v>100</v>
       </c>
-      <c r="E26" s="4">
+      <c r="E26" s="3">
         <v>83</v>
       </c>
-      <c r="F26" s="4">
+      <c r="F26" s="3">
         <v>95</v>
       </c>
-      <c r="G26" s="4">
+      <c r="G26" s="3">
         <v>74</v>
       </c>
-      <c r="H26" s="5">
+      <c r="H26" s="4">
         <f t="shared" si="0"/>
         <v>0.81200000000000006</v>
       </c>
@@ -1709,28 +1609,28 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A27" s="3">
+      <c r="A27" s="2">
         <v>26</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C27" s="4">
+      <c r="C27" s="3">
         <v>57</v>
       </c>
-      <c r="D27" s="4">
+      <c r="D27" s="3">
         <v>42</v>
       </c>
-      <c r="E27" s="4">
+      <c r="E27" s="3">
         <v>87</v>
       </c>
-      <c r="F27" s="4">
+      <c r="F27" s="3">
         <v>97</v>
       </c>
-      <c r="G27" s="4">
+      <c r="G27" s="3">
         <v>77</v>
       </c>
-      <c r="H27" s="5">
+      <c r="H27" s="4">
         <f t="shared" si="0"/>
         <v>0.72</v>
       </c>
@@ -1740,28 +1640,28 @@
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A28" s="3">
+      <c r="A28" s="2">
         <v>27</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="4">
+      <c r="C28" s="3">
         <v>60</v>
       </c>
-      <c r="D28" s="4">
+      <c r="D28" s="3">
         <v>47</v>
       </c>
-      <c r="E28" s="4">
+      <c r="E28" s="3">
         <v>91</v>
       </c>
-      <c r="F28" s="4">
+      <c r="F28" s="3">
         <v>99</v>
       </c>
-      <c r="G28" s="4">
+      <c r="G28" s="3">
         <v>80</v>
       </c>
-      <c r="H28" s="5">
+      <c r="H28" s="4">
         <f t="shared" si="0"/>
         <v>0.754</v>
       </c>
@@ -1771,28 +1671,28 @@
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A29" s="3">
+      <c r="A29" s="2">
         <v>28</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C29" s="4">
+      <c r="C29" s="3">
         <v>63</v>
       </c>
-      <c r="D29" s="4">
+      <c r="D29" s="3">
         <v>52</v>
       </c>
-      <c r="E29" s="4">
+      <c r="E29" s="3">
         <v>95</v>
       </c>
-      <c r="F29" s="4">
+      <c r="F29" s="3">
         <v>46</v>
       </c>
-      <c r="G29" s="4">
+      <c r="G29" s="3">
         <v>83</v>
       </c>
-      <c r="H29" s="5">
+      <c r="H29" s="4">
         <f t="shared" si="0"/>
         <v>0.67800000000000005</v>
       </c>
@@ -1802,28 +1702,28 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A30" s="3">
+      <c r="A30" s="2">
         <v>29</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C30" s="4">
+      <c r="C30" s="3">
         <v>66</v>
       </c>
-      <c r="D30" s="4">
+      <c r="D30" s="3">
         <v>57</v>
       </c>
-      <c r="E30" s="4">
+      <c r="E30" s="3">
         <v>99</v>
       </c>
-      <c r="F30" s="4">
+      <c r="F30" s="3">
         <v>48</v>
       </c>
-      <c r="G30" s="4">
+      <c r="G30" s="3">
         <v>86</v>
       </c>
-      <c r="H30" s="5">
+      <c r="H30" s="4">
         <f t="shared" si="0"/>
         <v>0.71199999999999997</v>
       </c>
@@ -1833,28 +1733,28 @@
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A31" s="3">
+      <c r="A31" s="2">
         <v>30</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C31" s="4">
+      <c r="C31" s="3">
         <v>69</v>
       </c>
-      <c r="D31" s="4">
+      <c r="D31" s="3">
         <v>62</v>
       </c>
-      <c r="E31" s="4">
+      <c r="E31" s="3">
         <v>44</v>
       </c>
-      <c r="F31" s="4">
+      <c r="F31" s="3">
         <v>50</v>
       </c>
-      <c r="G31" s="4">
+      <c r="G31" s="3">
         <v>89</v>
       </c>
-      <c r="H31" s="5">
+      <c r="H31" s="4">
         <f t="shared" si="0"/>
         <v>0.628</v>
       </c>
@@ -1864,28 +1764,28 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A32" s="3">
+      <c r="A32" s="2">
         <v>31</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="4">
+      <c r="C32" s="3">
         <v>72</v>
       </c>
-      <c r="D32" s="4">
+      <c r="D32" s="3">
         <v>67</v>
       </c>
-      <c r="E32" s="4">
+      <c r="E32" s="3">
         <v>48</v>
       </c>
-      <c r="F32" s="4">
+      <c r="F32" s="3">
         <v>52</v>
       </c>
-      <c r="G32" s="4">
+      <c r="G32" s="3">
         <v>92</v>
       </c>
-      <c r="H32" s="5">
+      <c r="H32" s="4">
         <f t="shared" si="0"/>
         <v>0.66200000000000003</v>
       </c>
@@ -1895,28 +1795,28 @@
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A33" s="3">
+      <c r="A33" s="2">
         <v>32</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C33" s="4">
+      <c r="C33" s="3">
         <v>75</v>
       </c>
-      <c r="D33" s="4">
+      <c r="D33" s="3">
         <v>72</v>
       </c>
-      <c r="E33" s="4">
+      <c r="E33" s="3">
         <v>52</v>
       </c>
-      <c r="F33" s="4">
+      <c r="F33" s="3">
         <v>54</v>
       </c>
-      <c r="G33" s="4">
+      <c r="G33" s="3">
         <v>95</v>
       </c>
-      <c r="H33" s="5">
+      <c r="H33" s="4">
         <f t="shared" si="0"/>
         <v>0.69599999999999995</v>
       </c>
@@ -1926,28 +1826,28 @@
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" s="3">
+      <c r="A34" s="2">
         <v>33</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C34" s="4">
+      <c r="C34" s="3">
         <v>78</v>
       </c>
-      <c r="D34" s="4">
+      <c r="D34" s="3">
         <v>77</v>
       </c>
-      <c r="E34" s="4">
+      <c r="E34" s="3">
         <v>56</v>
       </c>
-      <c r="F34" s="4">
+      <c r="F34" s="3">
         <v>56</v>
       </c>
-      <c r="G34" s="4">
+      <c r="G34" s="3">
         <v>98</v>
       </c>
-      <c r="H34" s="5">
+      <c r="H34" s="4">
         <f t="shared" si="0"/>
         <v>0.73</v>
       </c>
@@ -1957,28 +1857,28 @@
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A35" s="3">
+      <c r="A35" s="2">
         <v>34</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C35" s="4">
+      <c r="C35" s="3">
         <v>81</v>
       </c>
-      <c r="D35" s="4">
+      <c r="D35" s="3">
         <v>82</v>
       </c>
-      <c r="E35" s="4">
+      <c r="E35" s="3">
         <v>60</v>
       </c>
-      <c r="F35" s="4">
+      <c r="F35" s="3">
         <v>58</v>
       </c>
-      <c r="G35" s="4">
+      <c r="G35" s="3">
         <v>50</v>
       </c>
-      <c r="H35" s="5">
+      <c r="H35" s="4">
         <f t="shared" si="0"/>
         <v>0.66200000000000003</v>
       </c>
@@ -1988,28 +1888,28 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A36" s="3">
+      <c r="A36" s="2">
         <v>35</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C36" s="4">
+      <c r="C36" s="3">
         <v>84</v>
       </c>
-      <c r="D36" s="4">
+      <c r="D36" s="3">
         <v>87</v>
       </c>
-      <c r="E36" s="4">
+      <c r="E36" s="3">
         <v>64</v>
       </c>
-      <c r="F36" s="4">
+      <c r="F36" s="3">
         <v>60</v>
       </c>
-      <c r="G36" s="4">
+      <c r="G36" s="3">
         <v>53</v>
       </c>
-      <c r="H36" s="5">
+      <c r="H36" s="4">
         <f t="shared" si="0"/>
         <v>0.69599999999999995</v>
       </c>
@@ -2019,28 +1919,28 @@
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A37" s="3">
+      <c r="A37" s="2">
         <v>36</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C37" s="4">
+      <c r="C37" s="3">
         <v>87</v>
       </c>
-      <c r="D37" s="4">
+      <c r="D37" s="3">
         <v>92</v>
       </c>
-      <c r="E37" s="4">
+      <c r="E37" s="3">
         <v>68</v>
       </c>
-      <c r="F37" s="4">
+      <c r="F37" s="3">
         <v>62</v>
       </c>
-      <c r="G37" s="4">
+      <c r="G37" s="3">
         <v>56</v>
       </c>
-      <c r="H37" s="5">
+      <c r="H37" s="4">
         <f t="shared" si="0"/>
         <v>0.73</v>
       </c>
@@ -2050,28 +1950,28 @@
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A38" s="3">
+      <c r="A38" s="2">
         <v>37</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C38" s="4">
+      <c r="C38" s="3">
         <v>90</v>
       </c>
-      <c r="D38" s="4">
+      <c r="D38" s="3">
         <v>97</v>
       </c>
-      <c r="E38" s="4">
+      <c r="E38" s="3">
         <v>72</v>
       </c>
-      <c r="F38" s="4">
+      <c r="F38" s="3">
         <v>64</v>
       </c>
-      <c r="G38" s="4">
+      <c r="G38" s="3">
         <v>59</v>
       </c>
-      <c r="H38" s="5">
+      <c r="H38" s="4">
         <f t="shared" si="0"/>
         <v>0.76400000000000001</v>
       </c>
@@ -2081,28 +1981,28 @@
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A39" s="3">
+      <c r="A39" s="2">
         <v>38</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C39" s="4">
+      <c r="C39" s="3">
         <v>93</v>
       </c>
-      <c r="D39" s="4">
+      <c r="D39" s="3">
         <v>39</v>
       </c>
-      <c r="E39" s="4">
+      <c r="E39" s="3">
         <v>76</v>
       </c>
-      <c r="F39" s="4">
+      <c r="F39" s="3">
         <v>66</v>
       </c>
-      <c r="G39" s="4">
+      <c r="G39" s="3">
         <v>62</v>
       </c>
-      <c r="H39" s="5">
+      <c r="H39" s="4">
         <f t="shared" si="0"/>
         <v>0.67200000000000004</v>
       </c>
@@ -2112,28 +2012,28 @@
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A40" s="3">
+      <c r="A40" s="2">
         <v>39</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="B40" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C40" s="4">
+      <c r="C40" s="3">
         <v>96</v>
       </c>
-      <c r="D40" s="4">
+      <c r="D40" s="3">
         <v>44</v>
       </c>
-      <c r="E40" s="4">
+      <c r="E40" s="3">
         <v>80</v>
       </c>
-      <c r="F40" s="4">
+      <c r="F40" s="3">
         <v>68</v>
       </c>
-      <c r="G40" s="4">
+      <c r="G40" s="3">
         <v>65</v>
       </c>
-      <c r="H40" s="5">
+      <c r="H40" s="4">
         <f t="shared" si="0"/>
         <v>0.70599999999999996</v>
       </c>
@@ -2143,28 +2043,28 @@
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A41" s="3">
+      <c r="A41" s="2">
         <v>40</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="B41" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C41" s="4">
+      <c r="C41" s="3">
         <v>99</v>
       </c>
-      <c r="D41" s="4">
+      <c r="D41" s="3">
         <v>49</v>
       </c>
-      <c r="E41" s="4">
+      <c r="E41" s="3">
         <v>84</v>
       </c>
-      <c r="F41" s="4">
+      <c r="F41" s="3">
         <v>70</v>
       </c>
-      <c r="G41" s="4">
+      <c r="G41" s="3">
         <v>68</v>
       </c>
-      <c r="H41" s="5">
+      <c r="H41" s="4">
         <f t="shared" si="0"/>
         <v>0.74</v>
       </c>
@@ -2174,28 +2074,28 @@
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A42" s="3">
+      <c r="A42" s="2">
         <v>41</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="B42" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C42" s="4">
+      <c r="C42" s="3">
         <v>41</v>
       </c>
-      <c r="D42" s="4">
+      <c r="D42" s="3">
         <v>54</v>
       </c>
-      <c r="E42" s="4">
+      <c r="E42" s="3">
         <v>88</v>
       </c>
-      <c r="F42" s="4">
+      <c r="F42" s="3">
         <v>72</v>
       </c>
-      <c r="G42" s="4">
+      <c r="G42" s="3">
         <v>71</v>
       </c>
-      <c r="H42" s="5">
+      <c r="H42" s="4">
         <f t="shared" si="0"/>
         <v>0.65200000000000002</v>
       </c>
@@ -2205,28 +2105,28 @@
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A43" s="3">
+      <c r="A43" s="2">
         <v>42</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B43" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C43" s="4">
+      <c r="C43" s="3">
         <v>44</v>
       </c>
-      <c r="D43" s="4">
+      <c r="D43" s="3">
         <v>59</v>
       </c>
-      <c r="E43" s="4">
+      <c r="E43" s="3">
         <v>92</v>
       </c>
-      <c r="F43" s="4">
+      <c r="F43" s="3">
         <v>74</v>
       </c>
-      <c r="G43" s="4">
+      <c r="G43" s="3">
         <v>74</v>
       </c>
-      <c r="H43" s="5">
+      <c r="H43" s="4">
         <f t="shared" si="0"/>
         <v>0.68600000000000005</v>
       </c>
@@ -2236,28 +2136,28 @@
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A44" s="3">
+      <c r="A44" s="2">
         <v>43</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C44" s="4">
+      <c r="C44" s="3">
         <v>47</v>
       </c>
-      <c r="D44" s="4">
+      <c r="D44" s="3">
         <v>64</v>
       </c>
-      <c r="E44" s="4">
+      <c r="E44" s="3">
         <v>96</v>
       </c>
-      <c r="F44" s="4">
+      <c r="F44" s="3">
         <v>76</v>
       </c>
-      <c r="G44" s="4">
+      <c r="G44" s="3">
         <v>77</v>
       </c>
-      <c r="H44" s="5">
+      <c r="H44" s="4">
         <f t="shared" si="0"/>
         <v>0.72</v>
       </c>
@@ -2267,28 +2167,28 @@
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A45" s="3">
+      <c r="A45" s="2">
         <v>44</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C45" s="4">
+      <c r="C45" s="3">
         <v>50</v>
       </c>
-      <c r="D45" s="4">
+      <c r="D45" s="3">
         <v>69</v>
       </c>
-      <c r="E45" s="4">
+      <c r="E45" s="3">
         <v>100</v>
       </c>
-      <c r="F45" s="4">
+      <c r="F45" s="3">
         <v>78</v>
       </c>
-      <c r="G45" s="4">
+      <c r="G45" s="3">
         <v>80</v>
       </c>
-      <c r="H45" s="5">
+      <c r="H45" s="4">
         <f t="shared" si="0"/>
         <v>0.754</v>
       </c>
@@ -2298,28 +2198,28 @@
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A46" s="3">
+      <c r="A46" s="2">
         <v>45</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="B46" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C46" s="4">
+      <c r="C46" s="3">
         <v>53</v>
       </c>
-      <c r="D46" s="4">
+      <c r="D46" s="3">
         <v>74</v>
       </c>
-      <c r="E46" s="4">
+      <c r="E46" s="3">
         <v>45</v>
       </c>
-      <c r="F46" s="4">
+      <c r="F46" s="3">
         <v>80</v>
       </c>
-      <c r="G46" s="4">
+      <c r="G46" s="3">
         <v>83</v>
       </c>
-      <c r="H46" s="5">
+      <c r="H46" s="4">
         <f t="shared" si="0"/>
         <v>0.67</v>
       </c>
@@ -2329,28 +2229,28 @@
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A47" s="3">
+      <c r="A47" s="2">
         <v>46</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="B47" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C47" s="4">
+      <c r="C47" s="3">
         <v>56</v>
       </c>
-      <c r="D47" s="4">
+      <c r="D47" s="3">
         <v>79</v>
       </c>
-      <c r="E47" s="4">
+      <c r="E47" s="3">
         <v>49</v>
       </c>
-      <c r="F47" s="4">
+      <c r="F47" s="3">
         <v>82</v>
       </c>
-      <c r="G47" s="4">
+      <c r="G47" s="3">
         <v>86</v>
       </c>
-      <c r="H47" s="5">
+      <c r="H47" s="4">
         <f t="shared" si="0"/>
         <v>0.70399999999999996</v>
       </c>
@@ -2360,28 +2260,28 @@
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A48" s="3">
+      <c r="A48" s="2">
         <v>47</v>
       </c>
-      <c r="B48" s="3" t="s">
+      <c r="B48" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C48" s="4">
+      <c r="C48" s="3">
         <v>59</v>
       </c>
-      <c r="D48" s="4">
+      <c r="D48" s="3">
         <v>84</v>
       </c>
-      <c r="E48" s="4">
+      <c r="E48" s="3">
         <v>53</v>
       </c>
-      <c r="F48" s="4">
+      <c r="F48" s="3">
         <v>84</v>
       </c>
-      <c r="G48" s="4">
+      <c r="G48" s="3">
         <v>89</v>
       </c>
-      <c r="H48" s="5">
+      <c r="H48" s="4">
         <f t="shared" si="0"/>
         <v>0.73799999999999999</v>
       </c>
@@ -2391,28 +2291,28 @@
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A49" s="3">
+      <c r="A49" s="2">
         <v>48</v>
       </c>
-      <c r="B49" s="3" t="s">
+      <c r="B49" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C49" s="4">
+      <c r="C49" s="3">
         <v>62</v>
       </c>
-      <c r="D49" s="4">
+      <c r="D49" s="3">
         <v>89</v>
       </c>
-      <c r="E49" s="4">
+      <c r="E49" s="3">
         <v>57</v>
       </c>
-      <c r="F49" s="4">
+      <c r="F49" s="3">
         <v>86</v>
       </c>
-      <c r="G49" s="4">
+      <c r="G49" s="3">
         <v>92</v>
       </c>
-      <c r="H49" s="5">
+      <c r="H49" s="4">
         <f t="shared" si="0"/>
         <v>0.77200000000000002</v>
       </c>
@@ -2422,28 +2322,28 @@
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A50" s="3">
+      <c r="A50" s="2">
         <v>49</v>
       </c>
-      <c r="B50" s="3" t="s">
+      <c r="B50" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C50" s="4">
+      <c r="C50" s="3">
         <v>65</v>
       </c>
-      <c r="D50" s="4">
+      <c r="D50" s="3">
         <v>94</v>
       </c>
-      <c r="E50" s="4">
+      <c r="E50" s="3">
         <v>61</v>
       </c>
-      <c r="F50" s="4">
+      <c r="F50" s="3">
         <v>88</v>
       </c>
-      <c r="G50" s="4">
+      <c r="G50" s="3">
         <v>95</v>
       </c>
-      <c r="H50" s="5">
+      <c r="H50" s="4">
         <f t="shared" si="0"/>
         <v>0.80600000000000005</v>
       </c>
@@ -2453,28 +2353,28 @@
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A51" s="3">
+      <c r="A51" s="2">
         <v>50</v>
       </c>
-      <c r="B51" s="3" t="s">
+      <c r="B51" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C51" s="4">
+      <c r="C51" s="3">
         <v>68</v>
       </c>
-      <c r="D51" s="4">
+      <c r="D51" s="3">
         <v>99</v>
       </c>
-      <c r="E51" s="4">
+      <c r="E51" s="3">
         <v>65</v>
       </c>
-      <c r="F51" s="4">
+      <c r="F51" s="3">
         <v>90</v>
       </c>
-      <c r="G51" s="4">
+      <c r="G51" s="3">
         <v>98</v>
       </c>
-      <c r="H51" s="5">
+      <c r="H51" s="4">
         <f t="shared" si="0"/>
         <v>0.84</v>
       </c>
@@ -2484,27 +2384,18 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I51" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="C2:C51">
-    <cfRule type="cellIs" dxfId="7" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="7" operator="lessThan">
       <formula>60</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:G51">
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="6" operator="greaterThan">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I51">
-    <cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="fail">
-      <formula>NOT(ISERROR(SEARCH("fail",I2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="pass">
-      <formula>NOT(ISERROR(SEARCH("pass",I2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D2:D51">
-    <cfRule type="dataBar" priority="1">
+    <cfRule type="dataBar" priority="3">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -2515,6 +2406,35 @@
           <x14:id>{7FEEA0FB-4F00-4EDE-BEB6-321E425EEC1C}</x14:id>
         </ext>
       </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I51">
+    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="pass">
+      <formula>NOT(ISERROR(SEARCH("pass",I2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="fail">
+      <formula>NOT(ISERROR(SEARCH("fail",I2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E51">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F51">
+    <cfRule type="iconSet" priority="1">
+      <iconSet iconSet="3Symbols">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="33"/>
+        <cfvo type="percent" val="67"/>
+      </iconSet>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>